<commit_message>
feat: add payment methods report and Looker Studio dashboard integration
</commit_message>
<xml_diff>
--- a/reporte_mateando_datos.xlsx
+++ b/reporte_mateando_datos.xlsx
@@ -10,6 +10,7 @@
     <sheet name="Ventas Diarias" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Ranking Productos" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Resumen Estados" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Reporte Clientes y Pagos" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -829,4 +830,321 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E13"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>nombre_cliente</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>provincia</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>metodo_pago</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>total_pedidos</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>facturacion_total</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Federico Ruiz</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Mendoza</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Mercado Pago</t>
+        </is>
+      </c>
+      <c r="D2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E2" t="n">
+        <v>240000</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Carlos Pérez</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Córdoba</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Transferencia Bancaria</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>3</v>
+      </c>
+      <c r="E3" t="n">
+        <v>165000</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Sofía Martínez</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Buenos Aires</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Efectivo</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>1</v>
+      </c>
+      <c r="E4" t="n">
+        <v>160000</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Federico Ruiz</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Mendoza</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Tarjeta de Crédito</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>1</v>
+      </c>
+      <c r="E5" t="n">
+        <v>120000</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Mariana Benítez</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Santa Fe</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Mercado Pago</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>1</v>
+      </c>
+      <c r="E6" t="n">
+        <v>120000</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Sofía Martínez</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Buenos Aires</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Transferencia Bancaria</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>1</v>
+      </c>
+      <c r="E7" t="n">
+        <v>120000</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Federico Ruiz</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Mendoza</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Transferencia Bancaria</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>1</v>
+      </c>
+      <c r="E8" t="n">
+        <v>90000</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Sofía Martínez</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Buenos Aires</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Tarjeta de Crédito</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>1</v>
+      </c>
+      <c r="E9" t="n">
+        <v>90000</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Federico Ruiz</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Mendoza</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Efectivo</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>1</v>
+      </c>
+      <c r="E10" t="n">
+        <v>80000</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Mariana Benítez</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Santa Fe</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Transferencia Bancaria</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>1</v>
+      </c>
+      <c r="E11" t="n">
+        <v>60000</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Lucía Gómez</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Buenos Aires</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Efectivo</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>1</v>
+      </c>
+      <c r="E12" t="n">
+        <v>56000</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Lucía Gómez</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Buenos Aires</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Tarjeta de Crédito</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
+        <v>1</v>
+      </c>
+      <c r="E13" t="n">
+        <v>14000</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>